<commit_message>
Remove place, date and draft highlighting from FY 2025-26 financials
Drop the "Place: Bengaluru" and "Date:" lines from the signature blocks on
the Balance Sheet and the Statement of Profit and Loss, turn off the yellow
highlighting of open points, and remove the draft review sheet. The
statements are now 9 sheets / 10 printed pages with no draft markings.

Figures, captions, borders, fonts and layout are unchanged; the open points
remain recorded in the accompanying notes file.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015jSQaMdU8zCGZrHcENNREr
</commit_message>
<xml_diff>
--- a/Financials/Daivbharathi Technologies LLP/FY 2025-26/Daivbharathi_Technologies_LLP_Financials_FY_2025-26.xlsx
+++ b/Financials/Daivbharathi Technologies LLP/FY 2025-26/Daivbharathi_Technologies_LLP_Financials_FY_2025-26.xlsx
@@ -16,11 +16,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes 8-10" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes 11-12" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes 13-14" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open points - delete before use" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Balance Sheet'!$A$1:$F$74</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Profit and Loss'!$A$1:$F$66</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Balance Sheet'!$A$1:$F$70</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Profit and Loss'!$A$1:$F$62</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Notes 1-2 Policies'!$A$1:$F$79</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Note 3A-3B'!$A$1:$K$24</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Notes 4-5'!$A$1:$C$52</definedName>
@@ -28,7 +27,6 @@
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Notes 8-10'!$A$1:$D$53</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Notes 11-12'!$A$1:$C$67</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Notes 13-14'!$A$1:$F$25</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Open points - delete before use'!$A$1:$C$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -40,7 +38,7 @@
     <numFmt numFmtId="164" formatCode="[&gt;=100000]_(* ##\,##\,##0_);[&lt;=-100000]_(* \(##\,##\,##0\);_(* #,##0_)"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_)"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,17 +74,8 @@
       <b val="1"/>
       <sz val="7"/>
     </font>
-    <font>
-      <name val="Century Gothic"/>
-      <b val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Century Gothic"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -96,11 +85,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF99"/>
       </patternFill>
     </fill>
   </fills>
@@ -231,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -298,9 +282,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -358,13 +339,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -385,13 +360,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="3"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -406,7 +375,7 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -424,12 +393,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -437,9 +400,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -451,21 +411,6 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -832,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.97" customWidth="1" min="1" max="1"/>
@@ -1740,32 +1685,6 @@
       </c>
     </row>
     <row r="70" ht="9.75" customHeight="1"/>
-    <row r="71" ht="9.75" customHeight="1"/>
-    <row r="72" ht="9.75" customHeight="1">
-      <c r="A72" s="15" t="inlineStr">
-        <is>
-          <t>Place: Bengaluru</t>
-        </is>
-      </c>
-      <c r="C72" s="15" t="inlineStr">
-        <is>
-          <t>Place: Bengaluru</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="9.75" customHeight="1">
-      <c r="A73" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Date: </t>
-        </is>
-      </c>
-      <c r="C73" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Date: </t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="9.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="44">
     <mergeCell ref="B16:C16"/>
@@ -1818,283 +1737,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6.14" customWidth="1" min="1" max="1"/>
-    <col width="26.71" customWidth="1" min="2" max="2"/>
-    <col width="74.70999999999999" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="82" t="inlineStr">
-        <is>
-          <t>Draft for review - open points requiring confirmation (yellow cells in the statements refer to these points). Delete this sheet and remove the highlights once confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="9.75" customHeight="1"/>
-    <row r="3" ht="14" customHeight="1">
-      <c r="A3" s="83" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B3" s="83" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="C3" s="83" t="inlineStr">
-        <is>
-          <t>Point</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="79" customHeight="1">
-      <c r="A4" s="84" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B4" s="85" t="inlineStr">
-        <is>
-          <t>Partners' funds presentation</t>
-        </is>
-      </c>
-      <c r="C4" s="86" t="inlineStr">
-        <is>
-          <t>FY 2024-25 (signed) shows the loss allocated to the partners inside 'Partners Contribution' (Note 3A, 90:10) with Reserves &amp; Surplus nil. The FY 2025-26 statements show Partners' capital 90,000 and the accumulated loss (36,13,505) under Reserves &amp; Surplus (Note 2.2). The draft follows the FY 2025-26 presentation for the current year and shows the previous year exactly as signed. Please confirm which presentation to use for FY 2025-26. If the loss is to be allocated to partners (FY 2024-25 style), the partner-wise share of (24,92,591) at 90:10 does not divide into whole rupees - please provide the partner-wise figures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="41.5" customHeight="1">
-      <c r="A5" s="84" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B5" s="85" t="inlineStr">
-        <is>
-          <t>Opening balance of Reserves &amp; Surplus</t>
-        </is>
-      </c>
-      <c r="C5" s="86" t="inlineStr">
-        <is>
-          <t>Note 2.2 of the FY 2025-26 statements shows an opening balance of (11,20,914), whereas the FY 2024-25 loss as signed is (11,20,912) - a difference of Rs. 2. Both figures are retained as provided; please confirm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="54" customHeight="1">
-      <c r="A6" s="84" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B6" s="85" t="inlineStr">
-        <is>
-          <t>Partners' contribution 90,000 vs 1,00,000</t>
-        </is>
-      </c>
-      <c r="C6" s="86" t="inlineStr">
-        <is>
-          <t>FY 2024-25 shows contribution introduced 1,00,000 (Samartha 90,000 / Manasa 10,000) with 'Receivable From Partner' 10,000 in other current assets. FY 2025-26 shows contribution received 90,000 and no receivable. The FY 2025-26 statements do not give the partner-wise split, opening balance or amount introduced during the year (Note 2.1 B and D are blank) - these cells in Note 3A are left open (highlighted).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="66.5" customHeight="1">
-      <c r="A7" s="84" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B7" s="85" t="inlineStr">
-        <is>
-          <t>Classification of the loan (30,47,564)</t>
-        </is>
-      </c>
-      <c r="C7" s="86" t="inlineStr">
-        <is>
-          <t>FY 2024-25 classified the loan as Short-term borrowings - 'Loans and advances from related parties' (7,80,680). FY 2025-26 classifies 30,47,564 as Long-term borrowings - Unsecured - 'Loans and advances - Others' (Note 2.3), while Note 2.9 lists the same balance as a related-party balance. The draft keeps each year as provided (Note 5 long-term for FY 2025-26; Note 5A short-term for FY 2024-25). Please confirm the classification and caption.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="29" customHeight="1">
-      <c r="A8" s="84" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B8" s="85" t="inlineStr">
-        <is>
-          <t>Previous-year column</t>
-        </is>
-      </c>
-      <c r="C8" s="86" t="inlineStr">
-        <is>
-          <t>The FY 2025-26 statements have a single column. The draft fills the 'As at March 31, 2025' column from the signed FY 2024-25 statements. Confirm that comparatives are to be shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="91.5" customHeight="1">
-      <c r="A9" s="84" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B9" s="85" t="inlineStr">
-        <is>
-          <t>Note 12 - expense heads</t>
-        </is>
-      </c>
-      <c r="C9" s="86" t="inlineStr">
-        <is>
-          <t>The reference note uses fixed heads (Rent, Legal and professional charges, Printing and stationery, Communication expenses ...). The FY 2025-26 statements use 24 different heads. To avoid re-classifying, the draft keeps every FY 2025-26 head verbatim (highlighted) and only merges captions that are identical (Interest on TDS, Bank charges, Commission). Please confirm, or tell me which heads to merge (e.g. Advertisement -&gt; Advertisement and publicity; Printing charges -&gt; Printing and stationery; Telephone expenses -&gt; Communication expenses; Conveyance -&gt; Travelling expenses; Professional / consultancy / technical fees -&gt; Legal and professional charges).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="41.5" customHeight="1">
-      <c r="A10" s="84" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B10" s="85" t="inlineStr">
-        <is>
-          <t>Note 9 - cash captions</t>
-        </is>
-      </c>
-      <c r="C10" s="86" t="inlineStr">
-        <is>
-          <t>FY 2025-26 shows 'Balances with banks' 5,102, 'Cash on hand' 21,837 and 'Others' 18. The reference format has 'On current accounts'. The draft keeps the FY 2025-26 captions (highlighted). Confirm whether 'Balances with banks' should be shown as 'On current accounts', and the nature of 'Others' (Rs. 18).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="41.5" customHeight="1">
-      <c r="A11" s="84" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B11" s="85" t="inlineStr">
-        <is>
-          <t>Note 7 - Other current liabilities</t>
-        </is>
-      </c>
-      <c r="C11" s="86" t="inlineStr">
-        <is>
-          <t>The reference scan has the Note 7 heading but the table itself is missing (page 6). The draft uses the FY 2025-26 caption 'Other payables' 46,506 and shows the FY 2024-25 figure 35,000 on the same line - please confirm the FY 2024-25 break-up/caption.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="29" customHeight="1">
-      <c r="A12" s="84" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B12" s="85" t="inlineStr">
-        <is>
-          <t>Note 4 - movement rows</t>
-        </is>
-      </c>
-      <c r="C12" s="86" t="inlineStr">
-        <is>
-          <t>The reference shows only the closing balance. The draft adds the opening/loss/closing movement from Note 2.2 of the FY 2025-26 statements (highlighted). Confirm whether to keep or drop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="66.5" customHeight="1">
-      <c r="A13" s="84" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B13" s="85" t="inlineStr">
-        <is>
-          <t>Additional disclosures (Notes 13-14)</t>
-        </is>
-      </c>
-      <c r="C13" s="86" t="inlineStr">
-        <is>
-          <t>The FY 2025-26 statements contain a trade payables ageing schedule, a trade receivables ageing schedule (all nil), related-party disclosures, the partners' rights/duties paragraph and the MSME 45-day statement, none of which appear in the reference format. The draft includes the payables ageing and related-party notes as Notes 13-14 and the MSME statement under Note 6 (highlighted); the nil receivables ageing and the rights/duties paragraph are omitted. Confirm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="54" customHeight="1">
-      <c r="A14" s="84" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B14" s="85" t="inlineStr">
-        <is>
-          <t>Names and identifiers</t>
-        </is>
-      </c>
-      <c r="C14" s="86" t="inlineStr">
-        <is>
-          <t>The reference uses 'Samartha Raghava Nagabhushanam I' (trailing 'I'), 'Samartha R N', 'Manasa Nagabhushanam' and 'Manasa Nagabhushnam' in different places, and 'DIN'. The FY 2025-26 statements use 'MANASA NAGABHUSHNAM' and 'DPIN'. The draft replicates the reference text in each place. Please confirm the correct spellings.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="41.5" customHeight="1">
-      <c r="A15" s="84" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B15" s="85" t="inlineStr">
-        <is>
-          <t>Text corrections</t>
-        </is>
-      </c>
-      <c r="C15" s="86" t="inlineStr">
-        <is>
-          <t>The reference text is reproduced verbatim except for obvious typographical errors / duplicated words (incoporated, as flows, purcnase, thee, onon, duue, the garbled sentences in policies e, h and i, etc.). The full list is in the accompanying note. Tell me if you prefer the text exactly as in the reference.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="29" customHeight="1">
-      <c r="A16" s="84" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B16" s="85" t="inlineStr">
-        <is>
-          <t>Signing date</t>
-        </is>
-      </c>
-      <c r="C16" s="86" t="inlineStr">
-        <is>
-          <t>Place is kept as Bengaluru; the date on the Balance Sheet and P&amp;L is left blank.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="9.75" customHeight="1"/>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
-  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.8" customWidth="1" min="1" max="1"/>
@@ -2159,7 +1808,7 @@
     </row>
     <row r="8" ht="9.75" customHeight="1">
       <c r="A8" s="7" t="n"/>
-      <c r="F8" s="31" t="inlineStr">
+      <c r="F8" s="30" t="inlineStr">
         <is>
           <t>Amount in INR (Rs.)</t>
         </is>
@@ -2259,7 +1908,7 @@
           <t>III</t>
         </is>
       </c>
-      <c r="B14" s="32" t="inlineStr">
+      <c r="B14" s="31" t="inlineStr">
         <is>
           <t>Total revenue (I+II)</t>
         </is>
@@ -2269,7 +1918,7 @@
       <c r="E14" s="23" t="n">
         <v>1115272</v>
       </c>
-      <c r="F14" s="33" t="n">
+      <c r="F14" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2389,7 +2038,7 @@
     </row>
     <row r="23" ht="11.25" customHeight="1">
       <c r="A23" s="10" t="n"/>
-      <c r="B23" s="32" t="inlineStr">
+      <c r="B23" s="31" t="inlineStr">
         <is>
           <t>Total expenses</t>
         </is>
@@ -2416,17 +2065,17 @@
           <t>V</t>
         </is>
       </c>
-      <c r="B25" s="34" t="inlineStr">
+      <c r="B25" s="33" t="inlineStr">
         <is>
           <t>Profit / (Loss) before exceptional and extraordinary items,partners' remuneration and tax (III - IV)</t>
         </is>
       </c>
       <c r="C25" s="5" t="n"/>
       <c r="D25" s="5" t="n"/>
-      <c r="E25" s="35" t="n">
+      <c r="E25" s="34" t="n">
         <v>-2492591</v>
       </c>
-      <c r="F25" s="35" t="n">
+      <c r="F25" s="34" t="n">
         <v>-1120912</v>
       </c>
     </row>
@@ -2470,17 +2119,17 @@
           <t>VII</t>
         </is>
       </c>
-      <c r="B29" s="34" t="inlineStr">
+      <c r="B29" s="33" t="inlineStr">
         <is>
           <t>Profit / (Loss) before extraordinary items,partners' remuneration and tax (V - VI)</t>
         </is>
       </c>
       <c r="C29" s="5" t="n"/>
       <c r="D29" s="5" t="n"/>
-      <c r="E29" s="35" t="n">
+      <c r="E29" s="34" t="n">
         <v>-2492591</v>
       </c>
-      <c r="F29" s="35" t="n">
+      <c r="F29" s="34" t="n">
         <v>-1120912</v>
       </c>
     </row>
@@ -2531,10 +2180,10 @@
       </c>
       <c r="C33" s="5" t="n"/>
       <c r="D33" s="5" t="n"/>
-      <c r="E33" s="35" t="n">
+      <c r="E33" s="34" t="n">
         <v>-2492591</v>
       </c>
-      <c r="F33" s="35" t="n">
+      <c r="F33" s="34" t="n">
         <v>-1120912</v>
       </c>
     </row>
@@ -2581,10 +2230,10 @@
       </c>
       <c r="C37" s="5" t="n"/>
       <c r="D37" s="5" t="n"/>
-      <c r="E37" s="35" t="n">
+      <c r="E37" s="34" t="n">
         <v>-2492591</v>
       </c>
-      <c r="F37" s="35" t="n">
+      <c r="F37" s="34" t="n">
         <v>-1120912</v>
       </c>
     </row>
@@ -2667,10 +2316,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E43" s="35" t="n">
+      <c r="E43" s="34" t="n">
         <v>-2492591</v>
       </c>
-      <c r="F43" s="35" t="n">
+      <c r="F43" s="34" t="n">
         <v>-1120912</v>
       </c>
     </row>
@@ -2745,10 +2394,10 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E48" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" s="36" t="n">
+      <c r="E48" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2765,13 +2414,13 @@
           <t>XVII</t>
         </is>
       </c>
-      <c r="B50" s="32" t="inlineStr">
+      <c r="B50" s="31" t="inlineStr">
         <is>
           <t>Profit / (Loss) for the year (XI + XIV)</t>
         </is>
       </c>
       <c r="C50" s="22" t="n"/>
-      <c r="D50" s="37" t="inlineStr">
+      <c r="D50" s="36" t="inlineStr">
         <is>
           <t>A+B</t>
         </is>
@@ -2846,32 +2495,6 @@
       </c>
     </row>
     <row r="62" ht="9.75" customHeight="1"/>
-    <row r="63" ht="9.75" customHeight="1"/>
-    <row r="64" ht="9.75" customHeight="1">
-      <c r="A64" s="15" t="inlineStr">
-        <is>
-          <t>Place: Bengaluru</t>
-        </is>
-      </c>
-      <c r="C64" s="15" t="inlineStr">
-        <is>
-          <t>Place: Bengaluru</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="9.75" customHeight="1">
-      <c r="A65" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Date: </t>
-        </is>
-      </c>
-      <c r="C65" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Date: </t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="9.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="31">
     <mergeCell ref="B16:C16"/>
@@ -2929,14 +2552,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="12" customHeight="1">
-      <c r="A1" s="38" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Daivbharathi Technologies LLP</t>
         </is>
       </c>
     </row>
     <row r="2" ht="12" customHeight="1">
-      <c r="A2" s="38" t="inlineStr">
+      <c r="A2" s="37" t="inlineStr">
         <is>
           <t>Brief about the Firm and Significant Accounting policies for the year ended 31.03.2026</t>
         </is>
@@ -2944,14 +2567,14 @@
     </row>
     <row r="3" ht="9.75" customHeight="1"/>
     <row r="4" ht="12" customHeight="1">
-      <c r="B4" s="38" t="inlineStr">
+      <c r="B4" s="37" t="inlineStr">
         <is>
           <t>1.Brief about the Firm</t>
         </is>
       </c>
     </row>
     <row r="5" ht="34.5" customHeight="1">
-      <c r="B5" s="39" t="inlineStr">
+      <c r="B5" s="38" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2980,14 +2603,14 @@
     </row>
     <row r="6" ht="9.75" customHeight="1"/>
     <row r="7" ht="9.75" customHeight="1">
-      <c r="B7" s="40" t="inlineStr">
+      <c r="B7" s="39" t="inlineStr">
         <is>
           <t>The profit/loss sharing ratio as per the partnership deed is as follows:</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="B8" s="41" t="inlineStr">
+      <c r="B8" s="40" t="inlineStr">
         <is>
           <t>SR. NO</t>
         </is>
@@ -2999,7 +2622,7 @@
       </c>
       <c r="D8" s="10" t="n"/>
       <c r="E8" s="10" t="n"/>
-      <c r="F8" s="42" t="inlineStr">
+      <c r="F8" s="41" t="inlineStr">
         <is>
           <t>PERCENTAGE OF</t>
         </is>
@@ -3010,52 +2633,52 @@
       <c r="C9" s="10" t="n"/>
       <c r="D9" s="10" t="n"/>
       <c r="E9" s="10" t="n"/>
-      <c r="F9" s="42" t="inlineStr">
+      <c r="F9" s="41" t="inlineStr">
         <is>
           <t>PROFIT/LOSS</t>
         </is>
       </c>
     </row>
     <row r="10" ht="10.5" customHeight="1">
-      <c r="B10" s="43" t="inlineStr">
+      <c r="B10" s="42" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C10" s="43" t="inlineStr">
+      <c r="C10" s="42" t="inlineStr">
         <is>
           <t>Samartha Raghava Nagabhushanam</t>
         </is>
       </c>
       <c r="D10" s="10" t="n"/>
       <c r="E10" s="10" t="n"/>
-      <c r="F10" s="44" t="inlineStr">
+      <c r="F10" s="43" t="inlineStr">
         <is>
           <t>90%</t>
         </is>
       </c>
     </row>
     <row r="11" ht="10.5" customHeight="1">
-      <c r="B11" s="43" t="inlineStr">
+      <c r="B11" s="42" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="42" t="inlineStr">
         <is>
           <t>Manasa Nagabhushanam</t>
         </is>
       </c>
       <c r="D11" s="10" t="n"/>
       <c r="E11" s="10" t="n"/>
-      <c r="F11" s="44" t="inlineStr">
+      <c r="F11" s="43" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
     </row>
     <row r="12" ht="9.75" customHeight="1">
-      <c r="B12" s="40" t="inlineStr">
+      <c r="B12" s="39" t="inlineStr">
         <is>
           <t>Nature of Business:</t>
         </is>
@@ -3063,7 +2686,7 @@
     </row>
     <row r="13" ht="9.75" customHeight="1"/>
     <row r="14" ht="24" customHeight="1">
-      <c r="B14" s="39" t="inlineStr">
+      <c r="B14" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve"> To design and deploy innovative technological solutions that foster the spiritual growth and well-being of individuals, enabling them to lead more meaningful and fulfilling lives.</t>
         </is>
@@ -3072,7 +2695,7 @@
     <row r="15" ht="9.75" customHeight="1"/>
     <row r="16" ht="9.75" customHeight="1"/>
     <row r="17" ht="34.5" customHeight="1">
-      <c r="B17" s="39" t="inlineStr">
+      <c r="B17" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve"> To provide technology platforms and tools that facilitate the performance, preservation, and propagation of Hindu religious, cultural, and spiritual practices in alignment with traditional principles.</t>
         </is>
@@ -3082,7 +2705,7 @@
     <row r="19" ht="9.75" customHeight="1"/>
     <row r="20" ht="9.75" customHeight="1"/>
     <row r="21" ht="12" customHeight="1">
-      <c r="B21" s="38" t="inlineStr">
+      <c r="B21" s="37" t="inlineStr">
         <is>
           <t>2.SIGNIFICANT ACCOUNTING POLICIES</t>
         </is>
@@ -3090,7 +2713,7 @@
     </row>
     <row r="22" ht="9.75" customHeight="1"/>
     <row r="23" ht="12" customHeight="1">
-      <c r="B23" s="38" t="inlineStr">
+      <c r="B23" s="37" t="inlineStr">
         <is>
           <t>a.Basis of preparation The Financial Statements</t>
         </is>
@@ -3099,7 +2722,7 @@
     <row r="24" ht="9.75" customHeight="1"/>
     <row r="25" ht="9.75" customHeight="1"/>
     <row r="26" ht="45" customHeight="1">
-      <c r="B26" s="39" t="inlineStr">
+      <c r="B26" s="38" t="inlineStr">
         <is>
           <t>The Financial Statements have been prepared on accrual basis under historical cost convention and in accordance with the applicable accounting standards prescribed by the Institute of Chartered Accountants of India (ICAI). The accounting policies are consistently applied unless otherwise stated.</t>
         </is>
@@ -3108,7 +2731,7 @@
     <row r="27" ht="9.75" customHeight="1"/>
     <row r="28" ht="9.75" customHeight="1"/>
     <row r="29" ht="12" customHeight="1">
-      <c r="B29" s="38" t="inlineStr">
+      <c r="B29" s="37" t="inlineStr">
         <is>
           <t>b.Use of estimates</t>
         </is>
@@ -3117,7 +2740,7 @@
     <row r="30" ht="9.75" customHeight="1"/>
     <row r="31" ht="9.75" customHeight="1"/>
     <row r="32" ht="66" customHeight="1">
-      <c r="B32" s="39" t="inlineStr">
+      <c r="B32" s="38" t="inlineStr">
         <is>
           <t>The preparation of financial statements in conformity with generally accepted accounting principles requires management to make estimates and assumptions that affect the reported amount of revenue, expenses, assets and liabilities and the disclosure of contingent liabilities at the date of the financial statements and the results of operations during the reporting period end. Although these estimates are based upon management's best knowledge of current events and actions, actual results could differ from these estimates.</t>
         </is>
@@ -3126,7 +2749,7 @@
     <row r="33" ht="9.75" customHeight="1"/>
     <row r="34" ht="9.75" customHeight="1"/>
     <row r="35" ht="12" customHeight="1">
-      <c r="B35" s="38" t="inlineStr">
+      <c r="B35" s="37" t="inlineStr">
         <is>
           <t>c.Property, Plant &amp; Equipment Properties,</t>
         </is>
@@ -3135,7 +2758,7 @@
     <row r="36" ht="9.75" customHeight="1"/>
     <row r="37" ht="9.75" customHeight="1"/>
     <row r="38" ht="66" customHeight="1">
-      <c r="B38" s="39" t="inlineStr">
+      <c r="B38" s="38" t="inlineStr">
         <is>
           <t>Plant &amp; Equipment's are stated at cost less accumulated depreciation, amortization and impairment losses if any. Cost comprises the purchase price and any attributable cost of bringing the asset to its working condition for its intended use. Borrowing costs relating to acquisition of property, plant and equipment which takes substantial period of time to get ready for its intended use are also included to the extent they relate to the period till such assets are ready to be put to use.</t>
         </is>
@@ -3145,7 +2768,7 @@
     <row r="40" ht="9.75" customHeight="1"/>
     <row r="41" ht="9.75" customHeight="1"/>
     <row r="42" ht="34.5" customHeight="1">
-      <c r="B42" s="39" t="inlineStr">
+      <c r="B42" s="38" t="inlineStr">
         <is>
           <t>Depreciation on Property, Plant &amp; Equipment Depreciation on property, plant and equipment is provided on straight line method over the useful lives of assets except for leasehold improvements. Leasehold improvements are amortized over a period of 10 years.</t>
         </is>
@@ -3153,57 +2776,57 @@
     </row>
     <row r="43" ht="9.75" customHeight="1"/>
     <row r="44" ht="10.5" customHeight="1">
-      <c r="B44" s="44" t="inlineStr">
+      <c r="B44" s="43" t="inlineStr">
         <is>
           <t>Class of Assets</t>
         </is>
       </c>
       <c r="C44" s="10" t="n"/>
-      <c r="D44" s="45" t="inlineStr">
+      <c r="D44" s="44" t="inlineStr">
         <is>
           <t>Useful lives</t>
         </is>
       </c>
     </row>
     <row r="45" ht="10.5" customHeight="1">
-      <c r="B45" s="43" t="inlineStr">
+      <c r="B45" s="42" t="inlineStr">
         <is>
           <t>Office Equipment</t>
         </is>
       </c>
       <c r="C45" s="10" t="n"/>
-      <c r="D45" s="46" t="n">
+      <c r="D45" s="45" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="46" ht="10.5" customHeight="1">
-      <c r="B46" s="43" t="inlineStr">
+      <c r="B46" s="42" t="inlineStr">
         <is>
           <t>Computer</t>
         </is>
       </c>
       <c r="C46" s="10" t="n"/>
-      <c r="D46" s="46" t="n">
+      <c r="D46" s="45" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="47" ht="9.75" customHeight="1"/>
     <row r="48" ht="12" customHeight="1">
-      <c r="A48" s="38" t="inlineStr">
+      <c r="A48" s="37" t="inlineStr">
         <is>
           <t>Daivbharathi Technologies LLP</t>
         </is>
       </c>
     </row>
     <row r="49" ht="12" customHeight="1">
-      <c r="A49" s="38" t="inlineStr">
+      <c r="A49" s="37" t="inlineStr">
         <is>
           <t>Brief about the Firm and Significant Accounting policies for the year ended 31.03.2026</t>
         </is>
       </c>
     </row>
     <row r="50" ht="12" customHeight="1">
-      <c r="B50" s="38" t="inlineStr">
+      <c r="B50" s="37" t="inlineStr">
         <is>
           <t>d. Revenue recognition</t>
         </is>
@@ -3211,7 +2834,7 @@
     </row>
     <row r="51" ht="9.75" customHeight="1"/>
     <row r="52" ht="66" customHeight="1">
-      <c r="B52" s="39" t="inlineStr">
+      <c r="B52" s="38" t="inlineStr">
         <is>
           <t>Revenue is recognised to the extent that it is probable that the economic benefits will flow to the Firm and the amount of the revenue can be reliably measured with no uncertainty as regards to ultimate collection.
 Income from services:
@@ -3222,7 +2845,7 @@
     <row r="53" ht="9.75" customHeight="1"/>
     <row r="54" ht="9.75" customHeight="1"/>
     <row r="55" ht="12" customHeight="1">
-      <c r="B55" s="38" t="inlineStr">
+      <c r="B55" s="37" t="inlineStr">
         <is>
           <t>e.Investments</t>
         </is>
@@ -3230,7 +2853,7 @@
     </row>
     <row r="56" ht="9.75" customHeight="1"/>
     <row r="57" ht="55.5" customHeight="1">
-      <c r="B57" s="39" t="inlineStr">
+      <c r="B57" s="38" t="inlineStr">
         <is>
           <t>Investments that are readily realizable and intended to be held for not more than a year are classified as current investments. All other investments are classified as long-term investments. Current investments are carried at lower of cost and fair value determined on an individual investment basis. Long-term investments are carried at cost. However, provision for diminution in value is made to recognize a decline, other than temporary, in the value of the investments.</t>
         </is>
@@ -3239,7 +2862,7 @@
     <row r="58" ht="9.75" customHeight="1"/>
     <row r="59" ht="9.75" customHeight="1"/>
     <row r="60" ht="12" customHeight="1">
-      <c r="B60" s="38" t="inlineStr">
+      <c r="B60" s="37" t="inlineStr">
         <is>
           <t>f. Employee benefits</t>
         </is>
@@ -3247,7 +2870,7 @@
     </row>
     <row r="61" ht="9.75" customHeight="1"/>
     <row r="62" ht="108" customHeight="1">
-      <c r="B62" s="39" t="inlineStr">
+      <c r="B62" s="38" t="inlineStr">
         <is>
           <t>Defined contribution plans: Retirement benefits in the form of Provident Fund are a defined contribution scheme and the contributions are charged to the Statement of Profit and Loss of the year when the contributions to the fund is due. There are no other obligations other than the contribution payable to the fund. Defined benefit plans: Under Payment of Gratuity Act,1972 Gratuity liability is a defined benefit obligation and is provided for on the basis of an actuarial valuation on Projected Unit Credit Method made at the end of the financial year.  The Company records its gratuity liability based on an actuarial valuation made by an independent actuary as at year end. Compensated absences: Long term compensated absences are provided for based on actuarial valuation. The actuarial valuation is done as per Projected Unit Credit Method. All actuarial gains/losses are immediately taken to the Profit and Loss account and are not deferred.</t>
         </is>
@@ -3257,7 +2880,7 @@
     <row r="64" ht="9.75" customHeight="1"/>
     <row r="65" ht="9.75" customHeight="1"/>
     <row r="66" ht="12" customHeight="1">
-      <c r="B66" s="38" t="inlineStr">
+      <c r="B66" s="37" t="inlineStr">
         <is>
           <t>g.Cash and cash equivalents</t>
         </is>
@@ -3265,7 +2888,7 @@
     </row>
     <row r="67" ht="9.75" customHeight="1"/>
     <row r="68" ht="24" customHeight="1">
-      <c r="B68" s="39" t="inlineStr">
+      <c r="B68" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve"> Cash and cash equivalents in the Cash Flow Statement comprise cash at bank and in hand and short term investments with an original maturity of three months or less.</t>
         </is>
@@ -3275,7 +2898,7 @@
     <row r="70" ht="9.75" customHeight="1"/>
     <row r="71" ht="9.75" customHeight="1"/>
     <row r="72" ht="12" customHeight="1">
-      <c r="B72" s="38" t="inlineStr">
+      <c r="B72" s="37" t="inlineStr">
         <is>
           <t>h.Borrowing costs</t>
         </is>
@@ -3283,7 +2906,7 @@
     </row>
     <row r="73" ht="9.75" customHeight="1"/>
     <row r="74" ht="34.5" customHeight="1">
-      <c r="B74" s="39" t="inlineStr">
+      <c r="B74" s="38" t="inlineStr">
         <is>
           <t>Borrowing costs are recognized as an expense in the period in which these are incurred. Borrowing Costs that are attributable to the acquisition or construction of qualifying assets are capitalized as part of the cost of such assets.</t>
         </is>
@@ -3291,7 +2914,7 @@
     </row>
     <row r="75" ht="9.75" customHeight="1"/>
     <row r="76" ht="12" customHeight="1">
-      <c r="B76" s="38" t="inlineStr">
+      <c r="B76" s="37" t="inlineStr">
         <is>
           <t>i.Provisions</t>
         </is>
@@ -3299,7 +2922,7 @@
     </row>
     <row r="77" ht="9.75" customHeight="1"/>
     <row r="78" ht="66" customHeight="1">
-      <c r="B78" s="39" t="inlineStr">
+      <c r="B78" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve"> A provision is recognized when an enterprise has a present obligation as a result of past event; it is probable that an outflow of resources will be required to settle the obligation, in respect of which a reliable estimate can be made. Provisions are not discounted to its present value and are determined based on best estimate required to settle the obligation at the balance sheet date. These are reviewed at each balance sheet date and adjusted to reflect the current best estimates.</t>
         </is>
@@ -3390,7 +3013,7 @@
       <c r="K1" s="3" t="n"/>
     </row>
     <row r="2" ht="11" customHeight="1">
-      <c r="A2" s="47" t="inlineStr">
+      <c r="A2" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve"> DAIVBHARATHI TECHNOLOGIES LLP</t>
         </is>
@@ -3398,7 +3021,7 @@
       <c r="K2" s="5" t="n"/>
     </row>
     <row r="3" ht="11" customHeight="1">
-      <c r="A3" s="47" t="inlineStr">
+      <c r="A3" s="46" t="inlineStr">
         <is>
           <t>LLPIN: ACL-2422</t>
         </is>
@@ -3406,7 +3029,7 @@
       <c r="K3" s="5" t="n"/>
     </row>
     <row r="4" ht="11" customHeight="1">
-      <c r="A4" s="47" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t xml:space="preserve"> Notes forming part of the Financial Statements as at 31st March 2026</t>
         </is>
@@ -3418,7 +3041,7 @@
       <c r="K5" s="5" t="n"/>
     </row>
     <row r="6" ht="11" customHeight="1">
-      <c r="A6" s="47" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Note - 3A Partners Contribution Account</t>
         </is>
@@ -3427,7 +3050,7 @@
     </row>
     <row r="7" ht="9.75" customHeight="1">
       <c r="A7" s="7" t="n"/>
-      <c r="J7" s="48" t="inlineStr">
+      <c r="J7" s="47" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
@@ -3440,7 +3063,7 @@
           <t>3A</t>
         </is>
       </c>
-      <c r="B8" s="32" t="inlineStr">
+      <c r="B8" s="31" t="inlineStr">
         <is>
           <t>Partners Contribution Account</t>
         </is>
@@ -3518,7 +3141,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B10" s="49" t="inlineStr">
+      <c r="B10" s="48" t="inlineStr">
         <is>
           <t>Samartha R N</t>
         </is>
@@ -3526,13 +3149,13 @@
       <c r="C10" s="16" t="n">
         <v>90000</v>
       </c>
-      <c r="D10" s="31" t="inlineStr">
+      <c r="D10" s="30" t="inlineStr">
         <is>
           <t>90%</t>
         </is>
       </c>
-      <c r="E10" s="50" t="n"/>
-      <c r="F10" s="50" t="n"/>
+      <c r="E10" s="48" t="n"/>
+      <c r="F10" s="48" t="n"/>
       <c r="G10" s="17" t="n">
         <v>0</v>
       </c>
@@ -3542,10 +3165,10 @@
       <c r="I10" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="50" t="n"/>
+      <c r="J10" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="48" t="n"/>
     </row>
     <row r="11" ht="9.75" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
@@ -3553,7 +3176,7 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B11" s="49" t="inlineStr">
+      <c r="B11" s="48" t="inlineStr">
         <is>
           <t>Manasa Nagabhushnam</t>
         </is>
@@ -3561,13 +3184,13 @@
       <c r="C11" s="16" t="n">
         <v>10000</v>
       </c>
-      <c r="D11" s="31" t="inlineStr">
+      <c r="D11" s="30" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="E11" s="50" t="n"/>
-      <c r="F11" s="50" t="n"/>
+      <c r="E11" s="48" t="n"/>
+      <c r="F11" s="48" t="n"/>
       <c r="G11" s="17" t="n">
         <v>0</v>
       </c>
@@ -3577,28 +3200,28 @@
       <c r="I11" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="50" t="n"/>
+      <c r="J11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="48" t="n"/>
     </row>
     <row r="12" ht="10.5" customHeight="1">
       <c r="A12" s="11" t="n"/>
       <c r="B12" s="5" t="n"/>
       <c r="C12" s="5" t="n"/>
       <c r="D12" s="5" t="n"/>
-      <c r="E12" s="52" t="n"/>
-      <c r="F12" s="52" t="n"/>
-      <c r="G12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="33" t="n">
+      <c r="E12" s="49" t="n"/>
+      <c r="F12" s="49" t="n"/>
+      <c r="G12" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="32" t="n">
         <v>0</v>
       </c>
       <c r="K12" s="23" t="n">
@@ -3606,7 +3229,7 @@
       </c>
     </row>
     <row r="13" ht="10.5" customHeight="1">
-      <c r="A13" s="53" t="inlineStr">
+      <c r="A13" s="50" t="inlineStr">
         <is>
           <t>Previous Year (PY)</t>
         </is>
@@ -3614,39 +3237,39 @@
       <c r="B13" s="28" t="n"/>
       <c r="C13" s="28" t="n"/>
       <c r="D13" s="28" t="n"/>
-      <c r="E13" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="55" t="n">
+      <c r="E13" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="52" t="n">
         <v>100000</v>
       </c>
-      <c r="G13" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="55" t="n">
+      <c r="G13" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="52" t="n">
         <v>-1120912</v>
       </c>
-      <c r="K13" s="55" t="n">
+      <c r="K13" s="52" t="n">
         <v>-1020912</v>
       </c>
     </row>
     <row r="14" ht="9.75" customHeight="1"/>
     <row r="15" ht="9.75" customHeight="1"/>
     <row r="16" ht="11" customHeight="1">
-      <c r="A16" s="56" t="inlineStr">
+      <c r="A16" s="53" t="inlineStr">
         <is>
           <t>Note - 3B Partners Current Account</t>
         </is>
       </c>
     </row>
     <row r="17" ht="9.75" customHeight="1">
-      <c r="J17" s="48" t="inlineStr">
+      <c r="J17" s="47" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
@@ -3711,7 +3334,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B19" s="49" t="inlineStr">
+      <c r="B19" s="48" t="inlineStr">
         <is>
           <t>Samartha R N</t>
         </is>
@@ -3746,7 +3369,7 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B20" s="49" t="inlineStr">
+      <c r="B20" s="48" t="inlineStr">
         <is>
           <t>Manasa Nagabhushnam</t>
         </is>
@@ -3793,30 +3416,30 @@
       <c r="B22" s="5" t="n"/>
       <c r="C22" s="5" t="n"/>
       <c r="D22" s="5" t="n"/>
-      <c r="E22" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" s="33" t="n">
+      <c r="E22" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23" ht="9.75" customHeight="1">
-      <c r="A23" s="53" t="inlineStr">
+      <c r="A23" s="50" t="inlineStr">
         <is>
           <t>Previous Year (PY)</t>
         </is>
@@ -3824,25 +3447,25 @@
       <c r="B23" s="28" t="n"/>
       <c r="C23" s="28" t="n"/>
       <c r="D23" s="28" t="n"/>
-      <c r="E23" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="54" t="n">
+      <c r="E23" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="51" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3881,21 +3504,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="11.5" customHeight="1">
-      <c r="A1" s="38" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>DAIVBHARATHI TECHNOLOGIES LLP</t>
         </is>
       </c>
     </row>
     <row r="2" ht="11.5" customHeight="1">
-      <c r="A2" s="38" t="inlineStr">
+      <c r="A2" s="37" t="inlineStr">
         <is>
           <t>LLPIN: ACL-2422</t>
         </is>
       </c>
     </row>
     <row r="3" ht="11.5" customHeight="1">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="37" t="inlineStr">
         <is>
           <t>Notes forming part of the Financial Statements as at 31st March 2026</t>
         </is>
@@ -3903,12 +3526,12 @@
     </row>
     <row r="4" ht="9.75" customHeight="1"/>
     <row r="5" ht="11.5" customHeight="1">
-      <c r="A5" s="56" t="inlineStr">
+      <c r="A5" s="53" t="inlineStr">
         <is>
           <t>Note 4 : Reserves and Surplus</t>
         </is>
       </c>
-      <c r="C5" s="48" t="inlineStr">
+      <c r="C5" s="47" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
@@ -3934,7 +3557,7 @@
       </c>
     </row>
     <row r="7" ht="9.75" customHeight="1">
-      <c r="A7" s="57" t="inlineStr">
+      <c r="A7" s="54" t="inlineStr">
         <is>
           <t>Capital Reserve</t>
         </is>
@@ -3947,7 +3570,7 @@
       </c>
     </row>
     <row r="8" ht="9.75" customHeight="1">
-      <c r="A8" s="57" t="inlineStr">
+      <c r="A8" s="54" t="inlineStr">
         <is>
           <t>Revaluation Reserve</t>
         </is>
@@ -3960,7 +3583,7 @@
       </c>
     </row>
     <row r="9" ht="9.75" customHeight="1">
-      <c r="A9" s="57" t="inlineStr">
+      <c r="A9" s="54" t="inlineStr">
         <is>
           <t>Other Reserve</t>
         </is>
@@ -3973,7 +3596,7 @@
       </c>
     </row>
     <row r="10" ht="9.75" customHeight="1">
-      <c r="A10" s="57" t="inlineStr">
+      <c r="A10" s="54" t="inlineStr">
         <is>
           <t>Undistributed Surplus (Balance from statement of profit and loss)</t>
         </is>
@@ -3982,72 +3605,72 @@
       <c r="C10" s="5" t="n"/>
     </row>
     <row r="11" ht="9.75" customHeight="1">
-      <c r="A11" s="58" t="inlineStr">
+      <c r="A11" s="55" t="inlineStr">
         <is>
           <t>Opening Balance</t>
         </is>
       </c>
-      <c r="B11" s="59" t="n">
+      <c r="B11" s="16" t="n">
         <v>-1120914</v>
       </c>
-      <c r="C11" s="51" t="n">
+      <c r="C11" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12" ht="9.75" customHeight="1">
-      <c r="A12" s="58" t="inlineStr">
+      <c r="A12" s="55" t="inlineStr">
         <is>
           <t>Add: Profit/(Loss) for the year</t>
         </is>
       </c>
-      <c r="B12" s="59" t="n">
+      <c r="B12" s="16" t="n">
         <v>-2492591</v>
       </c>
-      <c r="C12" s="51" t="n">
+      <c r="C12" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13" ht="9.75" customHeight="1">
-      <c r="A13" s="58" t="inlineStr">
+      <c r="A13" s="55" t="inlineStr">
         <is>
           <t>Less: Amount utilised</t>
         </is>
       </c>
-      <c r="B13" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="51" t="n">
+      <c r="B13" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14" ht="9.75" customHeight="1">
-      <c r="A14" s="58" t="inlineStr">
+      <c r="A14" s="55" t="inlineStr">
         <is>
           <t>Less: Transfer to reserves</t>
         </is>
       </c>
-      <c r="B14" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="51" t="n">
+      <c r="B14" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15" ht="9.75" customHeight="1">
-      <c r="A15" s="58" t="inlineStr">
+      <c r="A15" s="55" t="inlineStr">
         <is>
           <t>Closing Balance</t>
         </is>
       </c>
-      <c r="B15" s="59" t="n">
+      <c r="B15" s="16" t="n">
         <v>-3613505</v>
       </c>
-      <c r="C15" s="51" t="n">
+      <c r="C15" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16" ht="9.75" customHeight="1">
-      <c r="A16" s="41" t="inlineStr">
+      <c r="A16" s="40" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -4055,19 +3678,19 @@
       <c r="B16" s="23" t="n">
         <v>-3613505</v>
       </c>
-      <c r="C16" s="33" t="n">
+      <c r="C16" s="32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17" ht="9.75" customHeight="1"/>
     <row r="18" ht="9.75" customHeight="1"/>
     <row r="19" ht="11.5" customHeight="1">
-      <c r="A19" s="56" t="inlineStr">
+      <c r="A19" s="53" t="inlineStr">
         <is>
           <t>Note 5 : Long-term borrowings</t>
         </is>
       </c>
-      <c r="C19" s="48" t="inlineStr">
+      <c r="C19" s="47" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
@@ -4093,20 +3716,20 @@
       </c>
     </row>
     <row r="21" ht="9.75" customHeight="1">
-      <c r="A21" s="60" t="inlineStr">
+      <c r="A21" s="56" t="inlineStr">
         <is>
           <t>Unsecured</t>
         </is>
       </c>
-      <c r="B21" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="36" t="n">
+      <c r="B21" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="35" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22" ht="9.75" customHeight="1">
-      <c r="A22" s="60" t="inlineStr">
+      <c r="A22" s="56" t="inlineStr">
         <is>
           <t>Term loans</t>
         </is>
@@ -4115,7 +3738,7 @@
       <c r="C22" s="5" t="n"/>
     </row>
     <row r="23" ht="9.75" customHeight="1">
-      <c r="A23" s="57" t="inlineStr">
+      <c r="A23" s="54" t="inlineStr">
         <is>
           <t>from banks</t>
         </is>
@@ -4124,7 +3747,7 @@
       <c r="C23" s="5" t="n"/>
     </row>
     <row r="24" ht="9.75" customHeight="1">
-      <c r="A24" s="57" t="inlineStr">
+      <c r="A24" s="54" t="inlineStr">
         <is>
           <t>from other parties</t>
         </is>
@@ -4138,7 +3761,7 @@
       <c r="C25" s="5" t="n"/>
     </row>
     <row r="26" ht="9.75" customHeight="1">
-      <c r="A26" s="60" t="inlineStr">
+      <c r="A26" s="56" t="inlineStr">
         <is>
           <t>Loans repayable on demand</t>
         </is>
@@ -4147,7 +3770,7 @@
       <c r="C26" s="5" t="n"/>
     </row>
     <row r="27" ht="9.75" customHeight="1">
-      <c r="A27" s="57" t="inlineStr">
+      <c r="A27" s="54" t="inlineStr">
         <is>
           <t>from banks</t>
         </is>
@@ -4160,7 +3783,7 @@
       </c>
     </row>
     <row r="28" ht="9.75" customHeight="1">
-      <c r="A28" s="57" t="inlineStr">
+      <c r="A28" s="54" t="inlineStr">
         <is>
           <t>from other parties</t>
         </is>
@@ -4173,7 +3796,7 @@
       </c>
     </row>
     <row r="29" ht="9.75" customHeight="1">
-      <c r="A29" s="57" t="inlineStr">
+      <c r="A29" s="54" t="inlineStr">
         <is>
           <t>Deferred payment liabilities</t>
         </is>
@@ -4186,7 +3809,7 @@
       </c>
     </row>
     <row r="30" ht="9.75" customHeight="1">
-      <c r="A30" s="57" t="inlineStr">
+      <c r="A30" s="54" t="inlineStr">
         <is>
           <t>Loans and advances from related parties</t>
         </is>
@@ -4199,20 +3822,20 @@
       </c>
     </row>
     <row r="31" ht="9.75" customHeight="1">
-      <c r="A31" s="61" t="inlineStr">
+      <c r="A31" s="54" t="inlineStr">
         <is>
           <t>Loans and advances - Others</t>
         </is>
       </c>
-      <c r="B31" s="59" t="n">
+      <c r="B31" s="16" t="n">
         <v>3047564</v>
       </c>
-      <c r="C31" s="51" t="n">
+      <c r="C31" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="32" ht="9.75" customHeight="1">
-      <c r="A32" s="57" t="inlineStr">
+      <c r="A32" s="54" t="inlineStr">
         <is>
           <t>Long term/current maturitites of finance lease obligation</t>
         </is>
@@ -4225,7 +3848,7 @@
       </c>
     </row>
     <row r="33" ht="9.75" customHeight="1">
-      <c r="A33" s="62" t="inlineStr">
+      <c r="A33" s="57" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -4233,19 +3856,19 @@
       <c r="B33" s="23" t="n">
         <v>3047564</v>
       </c>
-      <c r="C33" s="33" t="n">
+      <c r="C33" s="32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="34" ht="9.75" customHeight="1"/>
     <row r="35" ht="9.75" customHeight="1"/>
     <row r="36" ht="11.5" customHeight="1">
-      <c r="A36" s="56" t="inlineStr">
+      <c r="A36" s="53" t="inlineStr">
         <is>
           <t>Note 5A : Short-term borrowings</t>
         </is>
       </c>
-      <c r="C36" s="48" t="inlineStr">
+      <c r="C36" s="47" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
@@ -4271,20 +3894,20 @@
       </c>
     </row>
     <row r="38" ht="9.75" customHeight="1">
-      <c r="A38" s="60" t="inlineStr">
+      <c r="A38" s="56" t="inlineStr">
         <is>
           <t>Unsecured</t>
         </is>
       </c>
-      <c r="B38" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="C38" s="36" t="n">
+      <c r="B38" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="35" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="39" ht="9.75" customHeight="1">
-      <c r="A39" s="60" t="inlineStr">
+      <c r="A39" s="56" t="inlineStr">
         <is>
           <t>Term loans</t>
         </is>
@@ -4293,7 +3916,7 @@
       <c r="C39" s="5" t="n"/>
     </row>
     <row r="40" ht="9.75" customHeight="1">
-      <c r="A40" s="57" t="inlineStr">
+      <c r="A40" s="54" t="inlineStr">
         <is>
           <t>from banks</t>
         </is>
@@ -4302,7 +3925,7 @@
       <c r="C40" s="5" t="n"/>
     </row>
     <row r="41" ht="9.75" customHeight="1">
-      <c r="A41" s="57" t="inlineStr">
+      <c r="A41" s="54" t="inlineStr">
         <is>
           <t>from other parties</t>
         </is>
@@ -4316,7 +3939,7 @@
       <c r="C42" s="5" t="n"/>
     </row>
     <row r="43" ht="9.75" customHeight="1">
-      <c r="A43" s="60" t="inlineStr">
+      <c r="A43" s="56" t="inlineStr">
         <is>
           <t>Loans repayable on demand</t>
         </is>
@@ -4325,7 +3948,7 @@
       <c r="C43" s="5" t="n"/>
     </row>
     <row r="44" ht="9.75" customHeight="1">
-      <c r="A44" s="57" t="inlineStr">
+      <c r="A44" s="54" t="inlineStr">
         <is>
           <t>from banks</t>
         </is>
@@ -4338,7 +3961,7 @@
       </c>
     </row>
     <row r="45" ht="9.75" customHeight="1">
-      <c r="A45" s="57" t="inlineStr">
+      <c r="A45" s="54" t="inlineStr">
         <is>
           <t>from other parties</t>
         </is>
@@ -4351,7 +3974,7 @@
       </c>
     </row>
     <row r="46" ht="9.75" customHeight="1">
-      <c r="A46" s="57" t="inlineStr">
+      <c r="A46" s="54" t="inlineStr">
         <is>
           <t>Deferred payment liabilities</t>
         </is>
@@ -4364,20 +3987,20 @@
       </c>
     </row>
     <row r="47" ht="9.75" customHeight="1">
-      <c r="A47" s="57" t="inlineStr">
+      <c r="A47" s="54" t="inlineStr">
         <is>
           <t>Loans and advances from related parties</t>
         </is>
       </c>
-      <c r="B47" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="C47" s="59" t="n">
+      <c r="B47" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="16" t="n">
         <v>780680</v>
       </c>
     </row>
     <row r="48" ht="9.75" customHeight="1">
-      <c r="A48" s="57" t="inlineStr">
+      <c r="A48" s="54" t="inlineStr">
         <is>
           <t>Long term/current maturitites of finance lease obligation</t>
         </is>
@@ -4390,12 +4013,12 @@
       </c>
     </row>
     <row r="49" ht="9.75" customHeight="1">
-      <c r="A49" s="62" t="inlineStr">
+      <c r="A49" s="57" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B49" s="33" t="n">
+      <c r="B49" s="32" t="n">
         <v>0</v>
       </c>
       <c r="C49" s="23" t="n">
@@ -4431,21 +4054,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="11.5" customHeight="1">
-      <c r="A1" s="38" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>DAIVBHARATHI TECHNOLOGIES LLP</t>
         </is>
       </c>
     </row>
     <row r="2" ht="11.5" customHeight="1">
-      <c r="A2" s="38" t="inlineStr">
+      <c r="A2" s="37" t="inlineStr">
         <is>
           <t>LLPIN: ACL-2422</t>
         </is>
       </c>
     </row>
     <row r="3" ht="11.5" customHeight="1">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="37" t="inlineStr">
         <is>
           <t>Notes forming part of the Financial Statements as at 31st March 2026</t>
         </is>
@@ -4453,12 +4076,12 @@
     </row>
     <row r="4" ht="9.75" customHeight="1"/>
     <row r="5" ht="11.5" customHeight="1">
-      <c r="A5" s="56" t="inlineStr">
+      <c r="A5" s="53" t="inlineStr">
         <is>
           <t>Note 6 : Trade Payables</t>
         </is>
       </c>
-      <c r="C5" s="48" t="inlineStr">
+      <c r="C5" s="47" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
@@ -4484,7 +4107,7 @@
       </c>
     </row>
     <row r="7" ht="9.75" customHeight="1">
-      <c r="A7" s="57" t="inlineStr">
+      <c r="A7" s="54" t="inlineStr">
         <is>
           <t>Total outstanding dues of micro, small and medium enterprises</t>
         </is>
@@ -4497,7 +4120,7 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="63" t="inlineStr">
+      <c r="A8" s="58" t="inlineStr">
         <is>
           <t>Total outstanding dues of creditors other than micro, small and medium enterprises</t>
         </is>
@@ -4510,7 +4133,7 @@
       </c>
     </row>
     <row r="9" ht="9.75" customHeight="1">
-      <c r="A9" s="62" t="inlineStr">
+      <c r="A9" s="57" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -4551,7 +4174,7 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="63" t="inlineStr">
+      <c r="A14" s="58" t="inlineStr">
         <is>
           <t>(a) Amount remaining unpaid to any supplier at the end of each accounting year:</t>
         </is>
@@ -4560,7 +4183,7 @@
       <c r="C14" s="5" t="n"/>
     </row>
     <row r="15" ht="9.75" customHeight="1">
-      <c r="A15" s="57" t="inlineStr">
+      <c r="A15" s="54" t="inlineStr">
         <is>
           <t>-Principal</t>
         </is>
@@ -4573,7 +4196,7 @@
       </c>
     </row>
     <row r="16" ht="9.75" customHeight="1">
-      <c r="A16" s="57" t="inlineStr">
+      <c r="A16" s="54" t="inlineStr">
         <is>
           <t>-Interest</t>
         </is>
@@ -4586,20 +4209,20 @@
       </c>
     </row>
     <row r="17" ht="9.75" customHeight="1">
-      <c r="A17" s="60" t="inlineStr">
+      <c r="A17" s="56" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B17" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="33" t="n">
+      <c r="B17" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18" ht="31" customHeight="1">
-      <c r="A18" s="63" t="inlineStr">
+      <c r="A18" s="58" t="inlineStr">
         <is>
           <t>(b) The amount of interest paid by the buyer in terms of section 16 of the MSMED Act, along with the amount of the payment made to the supplier beyond the appointed day during each accounting year.</t>
         </is>
@@ -4612,7 +4235,7 @@
       </c>
     </row>
     <row r="19" ht="31" customHeight="1">
-      <c r="A19" s="63" t="inlineStr">
+      <c r="A19" s="58" t="inlineStr">
         <is>
           <t>(c) The amount of interest due and payable for the period of delay in making payment (which have been paid but beyond the appointed day during the year) but without adding the interest specified under the MSMED Act.</t>
         </is>
@@ -4625,7 +4248,7 @@
       </c>
     </row>
     <row r="20" ht="21" customHeight="1">
-      <c r="A20" s="63" t="inlineStr">
+      <c r="A20" s="58" t="inlineStr">
         <is>
           <t>(d) The amount of interest accrued and remaining unpaid at the end of each accounting year.</t>
         </is>
@@ -4638,21 +4261,21 @@
       </c>
     </row>
     <row r="21" ht="41" customHeight="1">
-      <c r="A21" s="64" t="inlineStr">
+      <c r="A21" s="59" t="inlineStr">
         <is>
           <t>(e) The amount of further interest remaining due and payable even in the succeeding years, until such date when the interest dues above are actually paid to the small enterprise, for the purpose of disallowance of a deductible expenditure under section 23 of the MSMED Act.</t>
         </is>
       </c>
-      <c r="B21" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="65" t="n">
+      <c r="B21" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="60" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22" ht="9.75" customHeight="1"/>
     <row r="23" ht="21" customHeight="1">
-      <c r="A23" s="66" t="inlineStr">
+      <c r="A23" s="61" t="inlineStr">
         <is>
           <t>There are no micro and small enterprises to which the LLP owes dues which are outstanding for more than 45 days as at the balance sheet date. Dues to Micro and Small Enterprises have been determined to the extent such parties have been identified on the basis of information available with the LLP.</t>
         </is>
@@ -4660,12 +4283,12 @@
     </row>
     <row r="24" ht="9.75" customHeight="1"/>
     <row r="25" ht="11.5" customHeight="1">
-      <c r="A25" s="56" t="inlineStr">
+      <c r="A25" s="53" t="inlineStr">
         <is>
           <t>Note 7 : Other current liabilities</t>
         </is>
       </c>
-      <c r="C25" s="48" t="inlineStr">
+      <c r="C25" s="47" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
@@ -4691,15 +4314,15 @@
       </c>
     </row>
     <row r="27" ht="9.75" customHeight="1">
-      <c r="A27" s="57" t="inlineStr">
+      <c r="A27" s="54" t="inlineStr">
         <is>
           <t>Other payables</t>
         </is>
       </c>
-      <c r="B27" s="59" t="n">
+      <c r="B27" s="16" t="n">
         <v>46506</v>
       </c>
-      <c r="C27" s="59" t="n">
+      <c r="C27" s="16" t="n">
         <v>35000</v>
       </c>
     </row>
@@ -4709,7 +4332,7 @@
       <c r="C28" s="5" t="n"/>
     </row>
     <row r="29" ht="9.75" customHeight="1">
-      <c r="A29" s="62" t="inlineStr">
+      <c r="A29" s="57" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -4753,21 +4376,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="11.5" customHeight="1">
-      <c r="A1" s="38" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Daivbharathi Technologies LLP</t>
         </is>
       </c>
     </row>
     <row r="2" ht="11.5" customHeight="1">
-      <c r="A2" s="38" t="inlineStr">
+      <c r="A2" s="37" t="inlineStr">
         <is>
           <t>LLPIN: ACL-2422</t>
         </is>
       </c>
     </row>
     <row r="3" ht="11.5" customHeight="1">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="37" t="inlineStr">
         <is>
           <t>Notes forming part of the Financial Statements as at March 31, 2026</t>
         </is>
@@ -4775,12 +4398,12 @@
     </row>
     <row r="4" ht="9.75" customHeight="1"/>
     <row r="5" ht="11.5" customHeight="1">
-      <c r="A5" s="56" t="inlineStr">
+      <c r="A5" s="53" t="inlineStr">
         <is>
           <t>Note 8 : Trade receivables</t>
         </is>
       </c>
-      <c r="D5" s="48" t="inlineStr">
+      <c r="D5" s="47" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
@@ -4807,7 +4430,7 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="67" t="inlineStr">
+      <c r="A7" s="62" t="inlineStr">
         <is>
           <t>Outstanding for a period less than 6 months from the date they are due for receipt</t>
         </is>
@@ -4817,7 +4440,7 @@
       <c r="D7" s="5" t="n"/>
     </row>
     <row r="8" ht="9.75" customHeight="1">
-      <c r="A8" s="68" t="inlineStr">
+      <c r="A8" s="63" t="inlineStr">
         <is>
           <t>Secured Considered good</t>
         </is>
@@ -4831,7 +4454,7 @@
       </c>
     </row>
     <row r="9" ht="9.75" customHeight="1">
-      <c r="A9" s="68" t="inlineStr">
+      <c r="A9" s="63" t="inlineStr">
         <is>
           <t>Unsecured Considered good</t>
         </is>
@@ -4845,7 +4468,7 @@
       </c>
     </row>
     <row r="10" ht="9.75" customHeight="1">
-      <c r="A10" s="68" t="inlineStr">
+      <c r="A10" s="63" t="inlineStr">
         <is>
           <t>Doubtful</t>
         </is>
@@ -4859,7 +4482,7 @@
       </c>
     </row>
     <row r="11" ht="9.75" customHeight="1">
-      <c r="A11" s="68" t="inlineStr">
+      <c r="A11" s="63" t="inlineStr">
         <is>
           <t>Less: Provision for doubtful receivables</t>
         </is>
@@ -4883,7 +4506,7 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="67" t="inlineStr">
+      <c r="A13" s="62" t="inlineStr">
         <is>
           <t>Outstanding for a period exceeding 6 months from the date they are due for receipt</t>
         </is>
@@ -4897,7 +4520,7 @@
       </c>
     </row>
     <row r="14" ht="9.75" customHeight="1">
-      <c r="A14" s="68" t="inlineStr">
+      <c r="A14" s="63" t="inlineStr">
         <is>
           <t>Secured Considered good</t>
         </is>
@@ -4911,7 +4534,7 @@
       </c>
     </row>
     <row r="15" ht="9.75" customHeight="1">
-      <c r="A15" s="68" t="inlineStr">
+      <c r="A15" s="63" t="inlineStr">
         <is>
           <t>Unsecured Considered good</t>
         </is>
@@ -4925,7 +4548,7 @@
       </c>
     </row>
     <row r="16" ht="9.75" customHeight="1">
-      <c r="A16" s="68" t="inlineStr">
+      <c r="A16" s="63" t="inlineStr">
         <is>
           <t>Doubtful</t>
         </is>
@@ -4939,7 +4562,7 @@
       </c>
     </row>
     <row r="17" ht="9.75" customHeight="1">
-      <c r="A17" s="68" t="inlineStr">
+      <c r="A17" s="63" t="inlineStr">
         <is>
           <t>Less: Provision for doubtful receivables</t>
         </is>
@@ -4953,7 +4576,7 @@
       </c>
     </row>
     <row r="18" ht="9.75" customHeight="1">
-      <c r="A18" s="68" t="inlineStr">
+      <c r="A18" s="63" t="inlineStr">
         <is>
           <t>Unbilled receivables</t>
         </is>
@@ -4977,28 +4600,28 @@
       </c>
     </row>
     <row r="20" ht="9.75" customHeight="1">
-      <c r="A20" s="69" t="inlineStr">
+      <c r="A20" s="64" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
       <c r="B20" s="22" t="n"/>
-      <c r="C20" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="33" t="n">
+      <c r="C20" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21" ht="9.75" customHeight="1"/>
     <row r="22" ht="9.75" customHeight="1"/>
     <row r="23" ht="11.5" customHeight="1">
-      <c r="A23" s="56" t="inlineStr">
+      <c r="A23" s="53" t="inlineStr">
         <is>
           <t>Note 9 : Cash and Bank Balances</t>
         </is>
       </c>
-      <c r="D23" s="48" t="inlineStr">
+      <c r="D23" s="47" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
@@ -5025,7 +4648,7 @@
       </c>
     </row>
     <row r="25" ht="9.75" customHeight="1">
-      <c r="A25" s="70" t="inlineStr">
+      <c r="A25" s="65" t="inlineStr">
         <is>
           <t>Cash and cash equivalents</t>
         </is>
@@ -5035,7 +4658,7 @@
       <c r="D25" s="5" t="n"/>
     </row>
     <row r="26" ht="9.75" customHeight="1">
-      <c r="A26" s="71" t="inlineStr">
+      <c r="A26" s="66" t="inlineStr">
         <is>
           <t>On current accounts</t>
         </is>
@@ -5049,21 +4672,21 @@
       </c>
     </row>
     <row r="27" ht="9.75" customHeight="1">
-      <c r="A27" s="72" t="inlineStr">
+      <c r="A27" s="66" t="inlineStr">
         <is>
           <t>Balances with banks</t>
         </is>
       </c>
       <c r="B27" s="5" t="n"/>
-      <c r="C27" s="59" t="n">
+      <c r="C27" s="16" t="n">
         <v>5102</v>
       </c>
-      <c r="D27" s="51" t="n">
+      <c r="D27" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28" ht="9.75" customHeight="1">
-      <c r="A28" s="68" t="inlineStr">
+      <c r="A28" s="63" t="inlineStr">
         <is>
           <t>Cash credit account (Debit balance)</t>
         </is>
@@ -5077,7 +4700,7 @@
       </c>
     </row>
     <row r="29" ht="9.75" customHeight="1">
-      <c r="A29" s="70" t="inlineStr">
+      <c r="A29" s="65" t="inlineStr">
         <is>
           <t>Fixed Deposits</t>
         </is>
@@ -5087,7 +4710,7 @@
       <c r="D29" s="5" t="n"/>
     </row>
     <row r="30" ht="9.75" customHeight="1">
-      <c r="A30" s="71" t="inlineStr">
+      <c r="A30" s="66" t="inlineStr">
         <is>
           <t>Deposits with original maturity of less than three months</t>
         </is>
@@ -5101,7 +4724,7 @@
       </c>
     </row>
     <row r="31" ht="9.75" customHeight="1">
-      <c r="A31" s="68" t="inlineStr">
+      <c r="A31" s="63" t="inlineStr">
         <is>
           <t>Cheques, drafts on hand</t>
         </is>
@@ -5115,7 +4738,7 @@
       </c>
     </row>
     <row r="32" ht="9.75" customHeight="1">
-      <c r="A32" s="68" t="inlineStr">
+      <c r="A32" s="63" t="inlineStr">
         <is>
           <t>Cash on hand</t>
         </is>
@@ -5129,26 +4752,26 @@
       </c>
     </row>
     <row r="33" ht="9.75" customHeight="1">
-      <c r="A33" s="73" t="inlineStr">
+      <c r="A33" s="63" t="inlineStr">
         <is>
           <t>Others</t>
         </is>
       </c>
       <c r="B33" s="5" t="n"/>
-      <c r="C33" s="59" t="n">
+      <c r="C33" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="D33" s="51" t="n">
+      <c r="D33" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="34" ht="9.75" customHeight="1">
-      <c r="A34" s="70" t="inlineStr">
+      <c r="A34" s="65" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B34" s="74" t="inlineStr">
+      <c r="B34" s="67" t="inlineStr">
         <is>
           <t>(I)</t>
         </is>
@@ -5167,7 +4790,7 @@
       <c r="D35" s="5" t="n"/>
     </row>
     <row r="36" ht="9.75" customHeight="1">
-      <c r="A36" s="70" t="inlineStr">
+      <c r="A36" s="65" t="inlineStr">
         <is>
           <t>Other bank balances</t>
         </is>
@@ -5177,7 +4800,7 @@
       <c r="D36" s="5" t="n"/>
     </row>
     <row r="37" ht="9.75" customHeight="1">
-      <c r="A37" s="68" t="inlineStr">
+      <c r="A37" s="63" t="inlineStr">
         <is>
           <t>Bank Deposits</t>
         </is>
@@ -5187,7 +4810,7 @@
       <c r="D37" s="5" t="n"/>
     </row>
     <row r="38" ht="9.75" customHeight="1">
-      <c r="A38" s="68" t="inlineStr">
+      <c r="A38" s="63" t="inlineStr">
         <is>
           <t>Earmarked Bank Deposits</t>
         </is>
@@ -5201,7 +4824,7 @@
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="67" t="inlineStr">
+      <c r="A39" s="62" t="inlineStr">
         <is>
           <t>Deposits with original maturity for more than 3 months but less than 12 months from reporting date</t>
         </is>
@@ -5215,7 +4838,7 @@
       </c>
     </row>
     <row r="40" ht="9.75" customHeight="1">
-      <c r="A40" s="68" t="inlineStr">
+      <c r="A40" s="63" t="inlineStr">
         <is>
           <t>Margin money or deposits under lien</t>
         </is>
@@ -5229,7 +4852,7 @@
       </c>
     </row>
     <row r="41" ht="9.75" customHeight="1">
-      <c r="A41" s="68" t="inlineStr">
+      <c r="A41" s="63" t="inlineStr">
         <is>
           <t>Others (specify nature)</t>
         </is>
@@ -5243,30 +4866,30 @@
       </c>
     </row>
     <row r="42" ht="9.75" customHeight="1">
-      <c r="A42" s="69" t="inlineStr">
+      <c r="A42" s="64" t="inlineStr">
         <is>
           <t>Total other bank balances</t>
         </is>
       </c>
-      <c r="B42" s="75" t="inlineStr">
+      <c r="B42" s="68" t="inlineStr">
         <is>
           <t>(II)</t>
         </is>
       </c>
-      <c r="C42" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D42" s="33" t="n">
+      <c r="C42" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="43" ht="9.75" customHeight="1">
-      <c r="A43" s="69" t="inlineStr">
+      <c r="A43" s="64" t="inlineStr">
         <is>
           <t>Total Cash and bank balances</t>
         </is>
       </c>
-      <c r="B43" s="75" t="inlineStr">
+      <c r="B43" s="68" t="inlineStr">
         <is>
           <t>(I+II)</t>
         </is>
@@ -5281,12 +4904,12 @@
     <row r="44" ht="9.75" customHeight="1"/>
     <row r="45" ht="9.75" customHeight="1"/>
     <row r="46" ht="11.5" customHeight="1">
-      <c r="A46" s="56" t="inlineStr">
+      <c r="A46" s="53" t="inlineStr">
         <is>
           <t>Note 10 Other Current Assets</t>
         </is>
       </c>
-      <c r="D46" s="48" t="inlineStr"/>
+      <c r="D46" s="47" t="inlineStr"/>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
@@ -5309,7 +4932,7 @@
       </c>
     </row>
     <row r="48" ht="9.75" customHeight="1">
-      <c r="A48" s="68" t="inlineStr">
+      <c r="A48" s="63" t="inlineStr">
         <is>
           <t>Receivable From Partner</t>
         </is>
@@ -5329,9 +4952,9 @@
       <c r="D49" s="5" t="n"/>
     </row>
     <row r="50" ht="9.75" customHeight="1">
-      <c r="A50" s="76" t="n"/>
+      <c r="A50" s="69" t="n"/>
       <c r="B50" s="28" t="n"/>
-      <c r="C50" s="33" t="n">
+      <c r="C50" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D50" s="23" t="n">
@@ -5401,21 +5024,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="11.5" customHeight="1">
-      <c r="A1" s="38" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Daivbharathi Technologies LLP</t>
         </is>
       </c>
     </row>
     <row r="2" ht="11.5" customHeight="1">
-      <c r="A2" s="38" t="inlineStr">
+      <c r="A2" s="37" t="inlineStr">
         <is>
           <t>LLPIN: ACL-2422</t>
         </is>
       </c>
     </row>
     <row r="3" ht="11.5" customHeight="1">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="37" t="inlineStr">
         <is>
           <t>Notes forming part of the Financial Statements as at 31st March 2026</t>
         </is>
@@ -5423,12 +5046,12 @@
     </row>
     <row r="4" ht="9.75" customHeight="1"/>
     <row r="5" ht="11.5" customHeight="1">
-      <c r="A5" s="56" t="inlineStr">
+      <c r="A5" s="53" t="inlineStr">
         <is>
           <t>Note 11: Revenue from operations</t>
         </is>
       </c>
-      <c r="C5" s="48" t="inlineStr">
+      <c r="C5" s="47" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
@@ -5454,7 +5077,7 @@
       </c>
     </row>
     <row r="7" ht="9.75" customHeight="1">
-      <c r="A7" s="57" t="inlineStr">
+      <c r="A7" s="54" t="inlineStr">
         <is>
           <t>Sale of products</t>
         </is>
@@ -5467,7 +5090,7 @@
       </c>
     </row>
     <row r="8" ht="9.75" customHeight="1">
-      <c r="A8" s="57" t="inlineStr">
+      <c r="A8" s="54" t="inlineStr">
         <is>
           <t>Sale of services</t>
         </is>
@@ -5480,7 +5103,7 @@
       </c>
     </row>
     <row r="9" ht="9.75" customHeight="1">
-      <c r="A9" s="57" t="inlineStr">
+      <c r="A9" s="54" t="inlineStr">
         <is>
           <t>Grants or donations received</t>
         </is>
@@ -5493,7 +5116,7 @@
       </c>
     </row>
     <row r="10" ht="9.75" customHeight="1">
-      <c r="A10" s="57" t="inlineStr">
+      <c r="A10" s="54" t="inlineStr">
         <is>
           <t>Other operating revenue</t>
         </is>
@@ -5506,7 +5129,7 @@
       </c>
     </row>
     <row r="11" ht="9.75" customHeight="1">
-      <c r="A11" s="62" t="inlineStr">
+      <c r="A11" s="57" t="inlineStr">
         <is>
           <t>Revenue from operations (Gross)</t>
         </is>
@@ -5514,12 +5137,12 @@
       <c r="B11" s="23" t="n">
         <v>1115272</v>
       </c>
-      <c r="C11" s="33" t="n">
+      <c r="C11" s="32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12" ht="9.75" customHeight="1">
-      <c r="A12" s="57" t="inlineStr">
+      <c r="A12" s="54" t="inlineStr">
         <is>
           <t>Less: Excise duty</t>
         </is>
@@ -5532,7 +5155,7 @@
       </c>
     </row>
     <row r="13" ht="9.75" customHeight="1">
-      <c r="A13" s="62" t="inlineStr">
+      <c r="A13" s="57" t="inlineStr">
         <is>
           <t>Revenue from operations (Net)</t>
         </is>
@@ -5540,19 +5163,19 @@
       <c r="B13" s="23" t="n">
         <v>1115272</v>
       </c>
-      <c r="C13" s="33" t="n">
+      <c r="C13" s="32" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14" ht="9.75" customHeight="1"/>
     <row r="15" ht="9.75" customHeight="1"/>
     <row r="16" ht="11.5" customHeight="1">
-      <c r="A16" s="56" t="inlineStr">
+      <c r="A16" s="53" t="inlineStr">
         <is>
           <t>Note 12: Other Expenses</t>
         </is>
       </c>
-      <c r="C16" s="48" t="inlineStr">
+      <c r="C16" s="47" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
@@ -5578,7 +5201,7 @@
       </c>
     </row>
     <row r="18" ht="9.75" customHeight="1">
-      <c r="A18" s="57" t="inlineStr">
+      <c r="A18" s="54" t="inlineStr">
         <is>
           <t>Consumption of stores and spare parts</t>
         </is>
@@ -5591,7 +5214,7 @@
       </c>
     </row>
     <row r="19" ht="9.75" customHeight="1">
-      <c r="A19" s="57" t="inlineStr">
+      <c r="A19" s="54" t="inlineStr">
         <is>
           <t>Interest on TDS</t>
         </is>
@@ -5604,7 +5227,7 @@
       </c>
     </row>
     <row r="20" ht="9.75" customHeight="1">
-      <c r="A20" s="57" t="inlineStr">
+      <c r="A20" s="54" t="inlineStr">
         <is>
           <t>Rent</t>
         </is>
@@ -5617,7 +5240,7 @@
       </c>
     </row>
     <row r="21" ht="9.75" customHeight="1">
-      <c r="A21" s="57" t="inlineStr">
+      <c r="A21" s="54" t="inlineStr">
         <is>
           <t>Repairs and maintenance - Buildings</t>
         </is>
@@ -5630,7 +5253,7 @@
       </c>
     </row>
     <row r="22" ht="9.75" customHeight="1">
-      <c r="A22" s="57" t="inlineStr">
+      <c r="A22" s="54" t="inlineStr">
         <is>
           <t>Repairs and maintenance - Machinery</t>
         </is>
@@ -5643,7 +5266,7 @@
       </c>
     </row>
     <row r="23" ht="9.75" customHeight="1">
-      <c r="A23" s="57" t="inlineStr">
+      <c r="A23" s="54" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
@@ -5656,7 +5279,7 @@
       </c>
     </row>
     <row r="24" ht="9.75" customHeight="1">
-      <c r="A24" s="57" t="inlineStr">
+      <c r="A24" s="54" t="inlineStr">
         <is>
           <t>Rent, Rates and taxes, excluding, taxes on income</t>
         </is>
@@ -5669,7 +5292,7 @@
       </c>
     </row>
     <row r="25" ht="9.75" customHeight="1">
-      <c r="A25" s="57" t="inlineStr">
+      <c r="A25" s="54" t="inlineStr">
         <is>
           <t>Labour charges</t>
         </is>
@@ -5682,7 +5305,7 @@
       </c>
     </row>
     <row r="26" ht="9.75" customHeight="1">
-      <c r="A26" s="57" t="inlineStr">
+      <c r="A26" s="54" t="inlineStr">
         <is>
           <t>Travelling expenses</t>
         </is>
@@ -5695,7 +5318,7 @@
       </c>
     </row>
     <row r="27" ht="9.75" customHeight="1">
-      <c r="A27" s="57" t="inlineStr">
+      <c r="A27" s="54" t="inlineStr">
         <is>
           <t>Auditor's remuneration (Refer note below)</t>
         </is>
@@ -5708,7 +5331,7 @@
       </c>
     </row>
     <row r="28" ht="9.75" customHeight="1">
-      <c r="A28" s="57" t="inlineStr">
+      <c r="A28" s="54" t="inlineStr">
         <is>
           <t>Printing and stationery</t>
         </is>
@@ -5721,7 +5344,7 @@
       </c>
     </row>
     <row r="29" ht="9.75" customHeight="1">
-      <c r="A29" s="57" t="inlineStr">
+      <c r="A29" s="54" t="inlineStr">
         <is>
           <t>Communication expenses</t>
         </is>
@@ -5734,7 +5357,7 @@
       </c>
     </row>
     <row r="30" ht="9.75" customHeight="1">
-      <c r="A30" s="57" t="inlineStr">
+      <c r="A30" s="54" t="inlineStr">
         <is>
           <t>Legal and professional charges</t>
         </is>
@@ -5747,7 +5370,7 @@
       </c>
     </row>
     <row r="31" ht="9.75" customHeight="1">
-      <c r="A31" s="57" t="inlineStr">
+      <c r="A31" s="54" t="inlineStr">
         <is>
           <t>Advertisement and publicity</t>
         </is>
@@ -5760,7 +5383,7 @@
       </c>
     </row>
     <row r="32" ht="9.75" customHeight="1">
-      <c r="A32" s="57" t="inlineStr">
+      <c r="A32" s="54" t="inlineStr">
         <is>
           <t>Bank Charges</t>
         </is>
@@ -5773,7 +5396,7 @@
       </c>
     </row>
     <row r="33" ht="9.75" customHeight="1">
-      <c r="A33" s="57" t="inlineStr">
+      <c r="A33" s="54" t="inlineStr">
         <is>
           <t>Business promotion expenses</t>
         </is>
@@ -5786,7 +5409,7 @@
       </c>
     </row>
     <row r="34" ht="9.75" customHeight="1">
-      <c r="A34" s="57" t="inlineStr">
+      <c r="A34" s="54" t="inlineStr">
         <is>
           <t>Commission</t>
         </is>
@@ -5799,7 +5422,7 @@
       </c>
     </row>
     <row r="35" ht="9.75" customHeight="1">
-      <c r="A35" s="57" t="inlineStr">
+      <c r="A35" s="54" t="inlineStr">
         <is>
           <t>Clearing and forwarding charges</t>
         </is>
@@ -5812,7 +5435,7 @@
       </c>
     </row>
     <row r="36" ht="9.75" customHeight="1">
-      <c r="A36" s="57" t="inlineStr">
+      <c r="A36" s="54" t="inlineStr">
         <is>
           <t>Loss on sale of Property, Plant and Equipment</t>
         </is>
@@ -5825,7 +5448,7 @@
       </c>
     </row>
     <row r="37" ht="9.75" customHeight="1">
-      <c r="A37" s="57" t="inlineStr">
+      <c r="A37" s="54" t="inlineStr">
         <is>
           <t>Loss on foreign exchange transactions (net)</t>
         </is>
@@ -5838,7 +5461,7 @@
       </c>
     </row>
     <row r="38" ht="9.75" customHeight="1">
-      <c r="A38" s="57" t="inlineStr">
+      <c r="A38" s="54" t="inlineStr">
         <is>
           <t>Loss on cancellation of forward contracts</t>
         </is>
@@ -5851,7 +5474,7 @@
       </c>
     </row>
     <row r="39" ht="9.75" customHeight="1">
-      <c r="A39" s="57" t="inlineStr">
+      <c r="A39" s="54" t="inlineStr">
         <is>
           <t>Loss on sale of investments (net)</t>
         </is>
@@ -5864,7 +5487,7 @@
       </c>
     </row>
     <row r="40" ht="9.75" customHeight="1">
-      <c r="A40" s="57" t="inlineStr">
+      <c r="A40" s="54" t="inlineStr">
         <is>
           <t>Provision for diminution in value of investments</t>
         </is>
@@ -5877,7 +5500,7 @@
       </c>
     </row>
     <row r="41" ht="9.75" customHeight="1">
-      <c r="A41" s="57" t="inlineStr">
+      <c r="A41" s="54" t="inlineStr">
         <is>
           <t>Provision for doubtful debts</t>
         </is>
@@ -5890,280 +5513,280 @@
       </c>
     </row>
     <row r="42" ht="9.75" customHeight="1">
-      <c r="A42" s="61" t="inlineStr">
+      <c r="A42" s="54" t="inlineStr">
         <is>
           <t>Accommodation and hotel expenses</t>
         </is>
       </c>
-      <c r="B42" s="59" t="n">
+      <c r="B42" s="16" t="n">
         <v>17510</v>
       </c>
-      <c r="C42" s="51" t="n">
+      <c r="C42" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="43" ht="9.75" customHeight="1">
-      <c r="A43" s="61" t="inlineStr">
+      <c r="A43" s="54" t="inlineStr">
         <is>
           <t>Advertisement</t>
         </is>
       </c>
-      <c r="B43" s="59" t="n">
+      <c r="B43" s="16" t="n">
         <v>410685</v>
       </c>
-      <c r="C43" s="51" t="n">
+      <c r="C43" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="44" ht="9.75" customHeight="1">
-      <c r="A44" s="61" t="inlineStr">
+      <c r="A44" s="54" t="inlineStr">
         <is>
           <t>Branding expenses</t>
         </is>
       </c>
-      <c r="B44" s="59" t="n">
+      <c r="B44" s="16" t="n">
         <v>19100</v>
       </c>
-      <c r="C44" s="51" t="n">
+      <c r="C44" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="45" ht="9.75" customHeight="1">
-      <c r="A45" s="61" t="inlineStr">
+      <c r="A45" s="54" t="inlineStr">
         <is>
           <t>Conveyance</t>
         </is>
       </c>
-      <c r="B45" s="59" t="n">
+      <c r="B45" s="16" t="n">
         <v>219790</v>
       </c>
-      <c r="C45" s="51" t="n">
+      <c r="C45" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="46" ht="9.75" customHeight="1">
-      <c r="A46" s="61" t="inlineStr">
+      <c r="A46" s="54" t="inlineStr">
         <is>
           <t>Data infrastructure expenses</t>
         </is>
       </c>
-      <c r="B46" s="59" t="n">
+      <c r="B46" s="16" t="n">
         <v>28583</v>
       </c>
-      <c r="C46" s="51" t="n">
+      <c r="C46" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="47" ht="9.75" customHeight="1">
-      <c r="A47" s="61" t="inlineStr">
+      <c r="A47" s="54" t="inlineStr">
         <is>
           <t>Design and development expenses</t>
         </is>
       </c>
-      <c r="B47" s="59" t="n">
+      <c r="B47" s="16" t="n">
         <v>75000</v>
       </c>
-      <c r="C47" s="51" t="n">
+      <c r="C47" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="48" ht="9.75" customHeight="1">
-      <c r="A48" s="61" t="inlineStr">
+      <c r="A48" s="54" t="inlineStr">
         <is>
           <t>GST late filing fees</t>
         </is>
       </c>
-      <c r="B48" s="59" t="n">
+      <c r="B48" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="C48" s="51" t="n">
+      <c r="C48" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="49" ht="9.75" customHeight="1">
-      <c r="A49" s="61" t="inlineStr">
+      <c r="A49" s="54" t="inlineStr">
         <is>
           <t>Internship charges</t>
         </is>
       </c>
-      <c r="B49" s="59" t="n">
+      <c r="B49" s="16" t="n">
         <v>36000</v>
       </c>
-      <c r="C49" s="51" t="n">
+      <c r="C49" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="50" ht="9.75" customHeight="1">
-      <c r="A50" s="61" t="inlineStr">
+      <c r="A50" s="54" t="inlineStr">
         <is>
           <t>Office expenses</t>
         </is>
       </c>
-      <c r="B50" s="59" t="n">
+      <c r="B50" s="16" t="n">
         <v>77518</v>
       </c>
-      <c r="C50" s="51" t="n">
+      <c r="C50" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="51" ht="9.75" customHeight="1">
-      <c r="A51" s="61" t="inlineStr">
+      <c r="A51" s="54" t="inlineStr">
         <is>
           <t>Pooja expenses</t>
         </is>
       </c>
-      <c r="B51" s="59" t="n">
+      <c r="B51" s="16" t="n">
         <v>1345327</v>
       </c>
-      <c r="C51" s="51" t="n">
+      <c r="C51" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="52" ht="9.75" customHeight="1">
-      <c r="A52" s="61" t="inlineStr">
+      <c r="A52" s="54" t="inlineStr">
         <is>
           <t>Pooja items</t>
         </is>
       </c>
-      <c r="B52" s="59" t="n">
+      <c r="B52" s="16" t="n">
         <v>50000</v>
       </c>
-      <c r="C52" s="51" t="n">
+      <c r="C52" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="53" ht="9.75" customHeight="1">
-      <c r="A53" s="61" t="inlineStr">
+      <c r="A53" s="54" t="inlineStr">
         <is>
           <t>Postage and courier expenses</t>
         </is>
       </c>
-      <c r="B53" s="59" t="n">
+      <c r="B53" s="16" t="n">
         <v>27286</v>
       </c>
-      <c r="C53" s="51" t="n">
+      <c r="C53" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="54" ht="9.75" customHeight="1">
-      <c r="A54" s="61" t="inlineStr">
+      <c r="A54" s="54" t="inlineStr">
         <is>
           <t>Pre-incorporation expenses</t>
         </is>
       </c>
-      <c r="B54" s="59" t="n">
+      <c r="B54" s="16" t="n">
         <v>36000</v>
       </c>
-      <c r="C54" s="51" t="n">
+      <c r="C54" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="55" ht="9.75" customHeight="1">
-      <c r="A55" s="61" t="inlineStr">
+      <c r="A55" s="54" t="inlineStr">
         <is>
           <t>Printing charges</t>
         </is>
       </c>
-      <c r="B55" s="59" t="n">
+      <c r="B55" s="16" t="n">
         <v>44706</v>
       </c>
-      <c r="C55" s="51" t="n">
+      <c r="C55" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="56" ht="9.75" customHeight="1">
-      <c r="A56" s="61" t="inlineStr">
+      <c r="A56" s="54" t="inlineStr">
         <is>
           <t>Professional / consultancy / technical fees</t>
         </is>
       </c>
-      <c r="B56" s="59" t="n">
+      <c r="B56" s="16" t="n">
         <v>1068252</v>
       </c>
-      <c r="C56" s="51" t="n">
+      <c r="C56" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="57" ht="9.75" customHeight="1">
-      <c r="A57" s="61" t="inlineStr">
+      <c r="A57" s="54" t="inlineStr">
         <is>
           <t>Staff welfare</t>
         </is>
       </c>
-      <c r="B57" s="59" t="n">
+      <c r="B57" s="16" t="n">
         <v>8021</v>
       </c>
-      <c r="C57" s="51" t="n">
+      <c r="C57" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="58" ht="9.75" customHeight="1">
-      <c r="A58" s="61" t="inlineStr">
+      <c r="A58" s="54" t="inlineStr">
         <is>
           <t>Studio expenses</t>
         </is>
       </c>
-      <c r="B58" s="59" t="n">
+      <c r="B58" s="16" t="n">
         <v>24000</v>
       </c>
-      <c r="C58" s="51" t="n">
+      <c r="C58" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="59" ht="9.75" customHeight="1">
-      <c r="A59" s="61" t="inlineStr">
+      <c r="A59" s="54" t="inlineStr">
         <is>
           <t>Subscription expenses</t>
         </is>
       </c>
-      <c r="B59" s="59" t="n">
+      <c r="B59" s="16" t="n">
         <v>15000</v>
       </c>
-      <c r="C59" s="51" t="n">
+      <c r="C59" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="60" ht="9.75" customHeight="1">
-      <c r="A60" s="61" t="inlineStr">
+      <c r="A60" s="54" t="inlineStr">
         <is>
           <t>Telephone expenses</t>
         </is>
       </c>
-      <c r="B60" s="59" t="n">
+      <c r="B60" s="16" t="n">
         <v>9871</v>
       </c>
-      <c r="C60" s="51" t="n">
+      <c r="C60" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="61" ht="9.75" customHeight="1">
-      <c r="A61" s="61" t="inlineStr">
+      <c r="A61" s="54" t="inlineStr">
         <is>
           <t>Translation expenses</t>
         </is>
       </c>
-      <c r="B61" s="59" t="n">
+      <c r="B61" s="16" t="n">
         <v>52760</v>
       </c>
-      <c r="C61" s="51" t="n">
+      <c r="C61" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="62" ht="9.75" customHeight="1">
-      <c r="A62" s="61" t="inlineStr">
+      <c r="A62" s="54" t="inlineStr">
         <is>
           <t>Website development expenses</t>
         </is>
       </c>
-      <c r="B62" s="59" t="n">
+      <c r="B62" s="16" t="n">
         <v>10000</v>
       </c>
-      <c r="C62" s="51" t="n">
+      <c r="C62" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="63" ht="9.75" customHeight="1">
-      <c r="A63" s="57" t="inlineStr">
+      <c r="A63" s="54" t="inlineStr">
         <is>
           <t>Miscellaneous expenses</t>
         </is>
@@ -6176,7 +5799,7 @@
       </c>
     </row>
     <row r="64" ht="9.75" customHeight="1">
-      <c r="A64" s="62" t="inlineStr">
+      <c r="A64" s="57" t="inlineStr">
         <is>
           <t>Total Other Expenses</t>
         </is>
@@ -6220,21 +5843,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="11.5" customHeight="1">
-      <c r="A1" s="38" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Daivbharathi Technologies LLP</t>
         </is>
       </c>
     </row>
     <row r="2" ht="11.5" customHeight="1">
-      <c r="A2" s="38" t="inlineStr">
+      <c r="A2" s="37" t="inlineStr">
         <is>
           <t>LLPIN: ACL-2422</t>
         </is>
       </c>
     </row>
     <row r="3" ht="11.5" customHeight="1">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="37" t="inlineStr">
         <is>
           <t>Notes forming part of the Financial Statements as at 31st March 2026</t>
         </is>
@@ -6242,19 +5865,19 @@
     </row>
     <row r="4" ht="9.75" customHeight="1"/>
     <row r="5" ht="11.5" customHeight="1">
-      <c r="A5" s="77" t="inlineStr">
+      <c r="A5" s="53" t="inlineStr">
         <is>
           <t>Note 13 : Trade Payables - Ageing schedule (Figures for the current reporting period)</t>
         </is>
       </c>
-      <c r="F5" s="48" t="inlineStr">
+      <c r="F5" s="47" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="12" customHeight="1">
-      <c r="A6" s="78" t="inlineStr">
+      <c r="A6" s="70" t="inlineStr">
         <is>
           <t>Particulars</t>
         </is>
@@ -6267,7 +5890,7 @@
       <c r="C6" s="10" t="n"/>
       <c r="D6" s="10" t="n"/>
       <c r="E6" s="10" t="n"/>
-      <c r="F6" s="78" t="inlineStr">
+      <c r="F6" s="70" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -6275,22 +5898,22 @@
     </row>
     <row r="7" ht="12" customHeight="1">
       <c r="A7" s="10" t="n"/>
-      <c r="B7" s="78" t="inlineStr">
+      <c r="B7" s="70" t="inlineStr">
         <is>
           <t>&lt; 1 Year</t>
         </is>
       </c>
-      <c r="C7" s="78" t="inlineStr">
+      <c r="C7" s="70" t="inlineStr">
         <is>
           <t>1-2 Years</t>
         </is>
       </c>
-      <c r="D7" s="78" t="inlineStr">
+      <c r="D7" s="70" t="inlineStr">
         <is>
           <t>2-3 Years</t>
         </is>
       </c>
-      <c r="E7" s="78" t="inlineStr">
+      <c r="E7" s="70" t="inlineStr">
         <is>
           <t>&gt; 3 Years</t>
         </is>
@@ -6298,7 +5921,7 @@
       <c r="F7" s="10" t="n"/>
     </row>
     <row r="8" ht="9.75" customHeight="1">
-      <c r="A8" s="57" t="inlineStr">
+      <c r="A8" s="54" t="inlineStr">
         <is>
           <t>MSME</t>
         </is>
@@ -6320,7 +5943,7 @@
       </c>
     </row>
     <row r="9" ht="9.75" customHeight="1">
-      <c r="A9" s="57" t="inlineStr">
+      <c r="A9" s="54" t="inlineStr">
         <is>
           <t>Others</t>
         </is>
@@ -6342,7 +5965,7 @@
       </c>
     </row>
     <row r="10" ht="9.75" customHeight="1">
-      <c r="A10" s="57" t="inlineStr">
+      <c r="A10" s="54" t="inlineStr">
         <is>
           <t>Disputed dues - MSME</t>
         </is>
@@ -6364,7 +5987,7 @@
       </c>
     </row>
     <row r="11" ht="9.75" customHeight="1">
-      <c r="A11" s="57" t="inlineStr">
+      <c r="A11" s="54" t="inlineStr">
         <is>
           <t>Disputed dues - Others</t>
         </is>
@@ -6386,7 +6009,7 @@
       </c>
     </row>
     <row r="12" ht="9.75" customHeight="1">
-      <c r="A12" s="62" t="inlineStr">
+      <c r="A12" s="57" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -6394,13 +6017,13 @@
       <c r="B12" s="23" t="n">
         <v>456392</v>
       </c>
-      <c r="C12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="33" t="n">
+      <c r="C12" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="32" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="23" t="n">
@@ -6410,7 +6033,7 @@
     <row r="13" ht="9.75" customHeight="1"/>
     <row r="14" ht="9.75" customHeight="1"/>
     <row r="15" ht="11.5" customHeight="1">
-      <c r="A15" s="77" t="inlineStr">
+      <c r="A15" s="53" t="inlineStr">
         <is>
           <t>Note 14 : Related Party Disclosures</t>
         </is>
@@ -6424,19 +6047,19 @@
       </c>
     </row>
     <row r="17" ht="12" customHeight="1">
-      <c r="A17" s="78" t="inlineStr">
+      <c r="A17" s="70" t="inlineStr">
         <is>
           <t>Sl No</t>
         </is>
       </c>
-      <c r="B17" s="78" t="inlineStr">
+      <c r="B17" s="70" t="inlineStr">
         <is>
           <t>Name of the Party</t>
         </is>
       </c>
       <c r="C17" s="10" t="n"/>
       <c r="D17" s="10" t="n"/>
-      <c r="E17" s="78" t="inlineStr">
+      <c r="E17" s="70" t="inlineStr">
         <is>
           <t>Name of relationship</t>
         </is>
@@ -6444,19 +6067,19 @@
       <c r="F17" s="10" t="n"/>
     </row>
     <row r="18" ht="9.75" customHeight="1">
-      <c r="A18" s="79" t="inlineStr">
+      <c r="A18" s="71" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B18" s="80" t="inlineStr">
+      <c r="B18" s="72" t="inlineStr">
         <is>
           <t>Samartha Raghava Nagabhushanam</t>
         </is>
       </c>
       <c r="C18" s="10" t="n"/>
       <c r="D18" s="10" t="n"/>
-      <c r="E18" s="80" t="inlineStr">
+      <c r="E18" s="72" t="inlineStr">
         <is>
           <t>Designated Partner</t>
         </is>
@@ -6464,19 +6087,19 @@
       <c r="F18" s="10" t="n"/>
     </row>
     <row r="19" ht="9.75" customHeight="1">
-      <c r="A19" s="79" t="inlineStr">
+      <c r="A19" s="71" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B19" s="80" t="inlineStr">
+      <c r="B19" s="72" t="inlineStr">
         <is>
           <t>Manasa Nagabhushnam</t>
         </is>
       </c>
       <c r="C19" s="10" t="n"/>
       <c r="D19" s="10" t="n"/>
-      <c r="E19" s="80" t="inlineStr">
+      <c r="E19" s="72" t="inlineStr">
         <is>
           <t>Designated Partner</t>
         </is>
@@ -6490,19 +6113,19 @@
           <t>b. Related Party Balances and Transactions:</t>
         </is>
       </c>
-      <c r="F21" s="48" t="inlineStr">
+      <c r="F21" s="47" t="inlineStr">
         <is>
           <t>(Amount in Rs.)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="78" t="inlineStr">
+      <c r="A22" s="70" t="inlineStr">
         <is>
           <t>Sl.No.</t>
         </is>
       </c>
-      <c r="B22" s="78" t="inlineStr">
+      <c r="B22" s="70" t="inlineStr">
         <is>
           <t>Nature of transaction</t>
         </is>
@@ -6518,37 +6141,37 @@
       <c r="F22" s="10" t="n"/>
     </row>
     <row r="23" ht="9.75" customHeight="1">
-      <c r="A23" s="79" t="inlineStr">
+      <c r="A23" s="71" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B23" s="80" t="inlineStr">
+      <c r="B23" s="72" t="inlineStr">
         <is>
           <t>Partners' capital contribution (closing balance)</t>
         </is>
       </c>
       <c r="C23" s="10" t="n"/>
       <c r="D23" s="10" t="n"/>
-      <c r="E23" s="81" t="n">
+      <c r="E23" s="73" t="n">
         <v>90000</v>
       </c>
       <c r="F23" s="10" t="n"/>
     </row>
     <row r="24" ht="9.75" customHeight="1">
-      <c r="A24" s="79" t="inlineStr">
+      <c r="A24" s="71" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B24" s="80" t="inlineStr">
+      <c r="B24" s="72" t="inlineStr">
         <is>
           <t>Unsecured loans - Others (closing balance)</t>
         </is>
       </c>
       <c r="C24" s="10" t="n"/>
       <c r="D24" s="10" t="n"/>
-      <c r="E24" s="81" t="n">
+      <c r="E24" s="73" t="n">
         <v>3047564</v>
       </c>
       <c r="F24" s="10" t="n"/>

</xml_diff>